<commit_message>
Add November budget explanation and email draft
Correct the PP-2611 Summary to Exclude VAT net amounts, keep the EcoVadis USD line out of the GBP totals, and include the humidity probe capex.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2611 Monthly Budget Application Form.xlsx
+++ b/2026/PP-2611 Monthly Budget Application Form.xlsx
@@ -5668,12 +5668,12 @@
         <v>0</v>
       </c>
       <c r="E4" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>8811.07</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>7342.56</v>
       </c>
       <c r="F4" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>20367.599999999999</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>16973</v>
       </c>
       <c r="G4" s="133">
         <f t="shared" ref="G4:G10" si="0">SUM(C4:D4)</f>
@@ -5681,7 +5681,7 @@
       </c>
       <c r="H4" s="143">
         <f t="shared" ref="H4:H10" si="1">SUM(E4:F4)</f>
-        <v>29178.67</v>
+        <v>24315.56</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
@@ -5691,27 +5691,27 @@
       </c>
       <c r="C5" s="135">
         <f>SUMIFS('Capex-A(Asset)'!$Q:$Q,'Capex-A(Asset)'!$D:$D,Summary!$B5,'Capex-A(Asset)'!$Z:$Z,C$3)</f>
-        <v>0</v>
+        <v>4507</v>
       </c>
       <c r="D5" s="136">
         <f>SUMIFS('Capex-A(Asset)'!$Q:$Q,'Capex-A(Asset)'!$D:$D,Summary!$B5,'Capex-A(Asset)'!$Z:$Z,D$3)</f>
         <v>0</v>
       </c>
       <c r="E5" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="F5" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1200</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>1000</v>
       </c>
       <c r="G5" s="133">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4507</v>
       </c>
       <c r="H5" s="143">
         <f t="shared" si="1"/>
-        <v>1200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1">
@@ -5728,11 +5728,11 @@
         <v>0</v>
       </c>
       <c r="E6" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="F6" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="G6" s="133">
@@ -5758,12 +5758,12 @@
         <v>0</v>
       </c>
       <c r="E7" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="F7" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1560</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>1300</v>
       </c>
       <c r="G7" s="133">
         <f t="shared" si="0"/>
@@ -5771,7 +5771,7 @@
       </c>
       <c r="H7" s="143">
         <f t="shared" si="1"/>
-        <v>1560</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
@@ -5788,11 +5788,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="F8" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="G8" s="133">
@@ -5818,12 +5818,12 @@
         <v>0</v>
       </c>
       <c r="E9" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>48548.076000000001</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>40456.73</v>
       </c>
       <c r="F9" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>36000</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>30000</v>
       </c>
       <c r="G9" s="133">
         <f t="shared" si="0"/>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="H9" s="143">
         <f t="shared" si="1"/>
-        <v>84548.076000000001</v>
+        <v>70456.73</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -5848,11 +5848,11 @@
         <v>0</v>
       </c>
       <c r="E10" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="F10" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="G10" s="133">
@@ -5880,11 +5880,11 @@
         <v>0</v>
       </c>
       <c r="E11" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B11,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>26742.400000000001</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B11,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
+        <v>20866</v>
       </c>
       <c r="F11" s="133">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B11,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B11,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
         <v>0</v>
       </c>
       <c r="G11" s="133">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="H11" s="143">
         <f t="shared" ref="H11" si="3">SUM(E11:F11)</f>
-        <v>26742.400000000001</v>
+        <v>20866</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1">
@@ -5902,28 +5902,28 @@
       </c>
       <c r="B12" s="178"/>
       <c r="C12" s="140">
-        <f t="shared" ref="C12:H12" si="4">SUM(C4:C10)</f>
-        <v>0</v>
+        <f>SUM(C4:C11)</f>
+        <v>4507</v>
       </c>
       <c r="D12" s="141">
-        <f t="shared" si="4"/>
+        <f>SUM(D4:D11)</f>
         <v>0</v>
       </c>
       <c r="E12" s="141">
         <f>SUM(E4:E11)</f>
-        <v>84101.546000000002</v>
+        <v>68665.29</v>
       </c>
       <c r="F12" s="141">
         <f>SUM(F4:F11)</f>
-        <v>59127.6</v>
+        <v>49273</v>
       </c>
       <c r="G12" s="140">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f>SUM(G4:G11)</f>
+        <v>4507</v>
       </c>
       <c r="H12" s="144">
         <f>SUM(H4:H11)</f>
-        <v>143229.14600000001</v>
+        <v>117938.29</v>
       </c>
     </row>
   </sheetData>
@@ -7980,7 +7980,9 @@
       </c>
       <c r="X4" s="80"/>
       <c r="Y4" s="84"/>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="52" t="s">
+        <v>7</v>
+      </c>
       <c r="AA4" s="86"/>
       <c r="AB4" s="87"/>
       <c r="AC4" s="96"/>

</xml_diff>

<commit_message>
Include acid dosing pump freight in the November budget
Add the £170 freight to the exclude-VAT pump amount and update the Summary, explanation, and application email.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2611 Monthly Budget Application Form.xlsx
+++ b/2026/PP-2611 Monthly Budget Application Form.xlsx
@@ -5819,7 +5819,7 @@
       </c>
       <c r="E9" s="133">
         <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
-        <v>40456.73</v>
+        <v>40626.73</v>
       </c>
       <c r="F9" s="133">
         <f>SUMIFS('K(Cost center)-Opex (Service)'!$Q:$Q,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3,'K(Cost center)-Opex (Service)'!$T:$T,"GBP")</f>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="H9" s="143">
         <f t="shared" si="1"/>
-        <v>70456.73</v>
+        <v>70626.73</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="E12" s="141">
         <f>SUM(E4:E11)</f>
-        <v>68665.29</v>
+        <v>68835.29</v>
       </c>
       <c r="F12" s="141">
         <f>SUM(F4:F11)</f>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="H12" s="144">
         <f>SUM(H4:H11)</f>
-        <v>117938.29</v>
+        <v>118108.29</v>
       </c>
     </row>
   </sheetData>
@@ -6176,16 +6176,16 @@
         <v>170</v>
       </c>
       <c r="Q4" s="123">
-        <f>O4*N4</f>
-        <v>16153.8</v>
+        <f>O4*N4+P4</f>
+        <v>16323.8</v>
       </c>
       <c r="R4" s="123">
         <f t="shared" ref="R4:R7" si="0">Q4*0.2</f>
-        <v>3230.76</v>
+        <v>3264.76</v>
       </c>
       <c r="S4" s="119">
         <f t="shared" ref="S4:S9" si="1">Q4+R4</f>
-        <v>19384.559999999998</v>
+        <v>19588.56</v>
       </c>
       <c r="T4" s="124" t="s">
         <v>56</v>

</xml_diff>